<commit_message>
feat: Implement Dynamic MLOps Model Registry and API Promotion
</commit_message>
<xml_diff>
--- a/data/raw/TPM.xlsx
+++ b/data/raw/TPM.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9584"/>
+  <dimension ref="A1:B9585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71006,6 +71006,14 @@
         <v>4.5</v>
       </c>
     </row>
+    <row r="9585">
+      <c r="A9585" s="1" t="n">
+        <v>46188.16666666666</v>
+      </c>
+      <c r="B9585" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix FFD Look-Ahead bias, update PSR calculation, fix trade entry timing in triple_barrera, and add EMBI lag
</commit_message>
<xml_diff>
--- a/data/raw/TPM.xlsx
+++ b/data/raw/TPM.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9585"/>
+  <dimension ref="A1:B9586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71014,6 +71014,14 @@
         <v>4.5</v>
       </c>
     </row>
+    <row r="9586">
+      <c r="A9586" s="1" t="n">
+        <v>46192.16666666666</v>
+      </c>
+      <c r="B9586" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>